<commit_message>
story-sheet-picker > staging: orders example with 7 sheets and 6 tables (counts differ)
Maintainer: raj-open <raj-open@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fake-sharepoint/library/Data/orders.xlsx
+++ b/tests/fake-sharepoint/library/Data/orders.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To do" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1144,4 +1145,39 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>order boxes for plums</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ask Hill Farm about pears</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
story-sheet-picker > staging: orders example with 6 sheets and 10 tables
- sheet Harvest: five small tables, one per week, each below its own title
- Suppliers and To do sheets dropped

Maintainer: raj-open <raj-open@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fake-sharepoint/library/Data/orders.xlsx
+++ b/tests/fake-sharepoint/library/Data/orders.xlsx
@@ -10,10 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harvest" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prices" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="To do" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -146,6 +145,17 @@
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="PriceList" displayName="PriceList" ref="B3:C8" headerRowCount="1">
+  <autoFilter ref="B3:C8"/>
+  <tableColumns count="2">
+    <tableColumn id="2" name="fruit"/>
+    <tableColumn id="3" name="price"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Regions" displayName="Regions" ref="F2:G5" headerRowCount="1">
   <autoFilter ref="F2:G5"/>
@@ -181,23 +191,60 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Suppliers" displayName="Suppliers" ref="B3:D6" headerRowCount="1">
-  <autoFilter ref="B3:D6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Week40" displayName="Week40" ref="B5:D7" headerRowCount="1">
+  <autoFilter ref="B5:D7"/>
   <tableColumns count="3">
-    <tableColumn id="2" name="supplier"/>
+    <tableColumn id="2" name="field"/>
     <tableColumn id="3" name="fruit"/>
-    <tableColumn id="4" name="since"/>
+    <tableColumn id="4" name="kg"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PriceList" displayName="PriceList" ref="B3:C8" headerRowCount="1">
-  <autoFilter ref="B3:C8"/>
-  <tableColumns count="2">
-    <tableColumn id="2" name="fruit"/>
-    <tableColumn id="3" name="price"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Week41" displayName="Week41" ref="B10:D12" headerRowCount="1">
+  <autoFilter ref="B10:D12"/>
+  <tableColumns count="3">
+    <tableColumn id="2" name="field"/>
+    <tableColumn id="3" name="fruit"/>
+    <tableColumn id="4" name="kg"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Week42" displayName="Week42" ref="B15:D17" headerRowCount="1">
+  <autoFilter ref="B15:D17"/>
+  <tableColumns count="3">
+    <tableColumn id="2" name="field"/>
+    <tableColumn id="3" name="fruit"/>
+    <tableColumn id="4" name="kg"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Week43" displayName="Week43" ref="B20:D22" headerRowCount="1">
+  <autoFilter ref="B20:D22"/>
+  <tableColumns count="3">
+    <tableColumn id="2" name="field"/>
+    <tableColumn id="3" name="fruit"/>
+    <tableColumn id="4" name="kg"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Week44" displayName="Week44" ref="B25:D27" headerRowCount="1">
+  <autoFilter ref="B25:D27"/>
+  <tableColumns count="3">
+    <tableColumn id="2" name="field"/>
+    <tableColumn id="3" name="fruit"/>
+    <tableColumn id="4" name="kg"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -931,89 +978,301 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:D6"/>
+  <dimension ref="B1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Suppliers</t>
+          <t>Harvest per week</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>contact by phone first</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>supplier</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>fruit</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>since</t>
+          <t>one table per week: field, fruit, kg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Orchard Lane</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>apple</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>2019</v>
+          <t>Week 40</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hill Farm</t>
+          <t>field</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pear</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>2022</v>
+          <t>fruit</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>Green Acres</t>
+          <t>north</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cherry</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Week 41</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fruit</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>banana</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>pear</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Week 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>fruit</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>cherry</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>plum</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>2024</v>
+      <c r="D17" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Week 43</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>fruit</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>pear</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Week 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>fruit</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>plum</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>banana</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
+  <tableParts count="5">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1145,39 +1404,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>to do</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>order boxes for plums</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ask Hill Farm about pears</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>